<commit_message>
Prestige index on SD-scaled indicators (Nobel Physics = 100); table notes as in the paper (summary statistics, prize list, early-career list, robustness, awarding countries, home-bias prizes); rTwoOneMultiCriteria no longer a paper macro; expected/ refreshed
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cleanPrizeList.xlsx
+++ b/data/cleanPrizeList.xlsx
@@ -786,7 +786,7 @@
         <v>0.453135606863188</v>
       </c>
       <c r="AK2" t="n">
-        <v>4.608937589932658</v>
+        <v>9.641353842442056</v>
       </c>
       <c r="AL2" t="n">
         <v>100</v>
@@ -804,7 +804,7 @@
         <v>2.756878863437439</v>
       </c>
       <c r="AQ2" t="n">
-        <v>3.710313977089529</v>
+        <v>8.855471272811485</v>
       </c>
       <c r="AR2" t="n">
         <v>100</v>
@@ -946,10 +946,10 @@
         <v>0.4002480057170862</v>
       </c>
       <c r="AK3" t="n">
-        <v>4.34022189683815</v>
+        <v>9.372638149347546</v>
       </c>
       <c r="AL3" t="n">
-        <v>94.1696825385211</v>
+        <v>97.21288423300469</v>
       </c>
       <c r="AM3" t="n">
         <v>2</v>
@@ -964,10 +964,10 @@
         <v>2.578938588925572</v>
       </c>
       <c r="AQ3" t="n">
-        <v>3.518132412887604</v>
+        <v>8.663289708609559</v>
       </c>
       <c r="AR3" t="n">
-        <v>94.82034228400592</v>
+        <v>97.82979856993076</v>
       </c>
       <c r="AS3" t="n">
         <v>3</v>
@@ -1106,10 +1106,10 @@
         <v>0.4640582914922362</v>
       </c>
       <c r="AK4" t="n">
-        <v>4.290327687732292</v>
+        <v>9.32274394024169</v>
       </c>
       <c r="AL4" t="n">
-        <v>93.08712917058567</v>
+        <v>96.69538212778978</v>
       </c>
       <c r="AM4" t="n">
         <v>3</v>
@@ -1124,10 +1124,10 @@
         <v>2.462883935525228</v>
       </c>
       <c r="AQ4" t="n">
-        <v>3.522698862984222</v>
+        <v>8.667856158706178</v>
       </c>
       <c r="AR4" t="n">
-        <v>94.94341677648325</v>
+        <v>97.88136499656058</v>
       </c>
       <c r="AS4" t="n">
         <v>2</v>
@@ -1262,10 +1262,10 @@
         <v>0.4462586499025186</v>
       </c>
       <c r="AK5" t="n">
-        <v>4.24722431047303</v>
+        <v>9.279640562982427</v>
       </c>
       <c r="AL5" t="n">
-        <v>92.15191630605452</v>
+        <v>96.24831444451986</v>
       </c>
       <c r="AM5" t="n">
         <v>4</v>
@@ -1280,10 +1280,10 @@
         <v>2.579974131782145</v>
       </c>
       <c r="AQ5" t="n">
-        <v>3.411465612116208</v>
+        <v>8.556622907838163</v>
       </c>
       <c r="AR5" t="n">
-        <v>91.94546966055563</v>
+        <v>96.62526865294159</v>
       </c>
       <c r="AS5" t="n">
         <v>4</v>
@@ -1418,10 +1418,10 @@
         <v>0.459201694756012</v>
       </c>
       <c r="AK6" t="n">
-        <v>3.587475763076701</v>
+        <v>8.6198920155861</v>
       </c>
       <c r="AL6" t="n">
-        <v>77.83736909158534</v>
+        <v>89.40541086294961</v>
       </c>
       <c r="AM6" t="n">
         <v>5</v>
@@ -1436,10 +1436,10 @@
         <v>1.694014129546979</v>
       </c>
       <c r="AQ6" t="n">
-        <v>3.182647120570222</v>
+        <v>8.327804416292176</v>
       </c>
       <c r="AR6" t="n">
-        <v>85.77837725385109</v>
+        <v>94.04134641439832</v>
       </c>
       <c r="AS6" t="n">
         <v>5</v>
@@ -1574,10 +1574,10 @@
         <v>0.4206237754852382</v>
       </c>
       <c r="AK7" t="n">
-        <v>3.429962881584475</v>
+        <v>8.462379134093872</v>
       </c>
       <c r="AL7" t="n">
-        <v>74.41981616493511</v>
+        <v>87.77168925013169</v>
       </c>
       <c r="AM7" t="n">
         <v>6</v>
@@ -1592,10 +1592,10 @@
         <v>2.13402030478669</v>
       </c>
       <c r="AQ7" t="n">
-        <v>2.66374895303703</v>
+        <v>7.808906248758986</v>
       </c>
       <c r="AR7" t="n">
-        <v>71.79308730973078</v>
+        <v>88.18171284383571</v>
       </c>
       <c r="AS7" t="n">
         <v>7</v>
@@ -1730,10 +1730,10 @@
         <v>0.5045057590475742</v>
       </c>
       <c r="AK8" t="n">
-        <v>3.183972193534811</v>
+        <v>8.216388446044208</v>
       </c>
       <c r="AL8" t="n">
-        <v>69.08256255171666</v>
+        <v>85.22027694777647</v>
       </c>
       <c r="AM8" t="n">
         <v>7</v>
@@ -1748,10 +1748,10 @@
         <v>1.206770912210374</v>
       </c>
       <c r="AQ8" t="n">
-        <v>3.035033524787963</v>
+        <v>8.180190820509919</v>
       </c>
       <c r="AR8" t="n">
-        <v>81.7999108304232</v>
+        <v>92.37442670753339</v>
       </c>
       <c r="AS8" t="n">
         <v>6</v>
@@ -1886,10 +1886,10 @@
         <v>0.3832985146851033</v>
       </c>
       <c r="AK9" t="n">
-        <v>1.545883417686152</v>
+        <v>6.578299670195549</v>
       </c>
       <c r="AL9" t="n">
-        <v>33.54099263706321</v>
+        <v>68.23004090190443</v>
       </c>
       <c r="AM9" t="n">
         <v>8</v>
@@ -1904,10 +1904,10 @@
         <v>1.438058539948469</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.9186656525270754</v>
+        <v>6.063822948249031</v>
       </c>
       <c r="AR9" t="n">
-        <v>24.75978200765914</v>
+        <v>68.47544034010349</v>
       </c>
       <c r="AS9" t="n">
         <v>15</v>
@@ -2042,10 +2042,10 @@
         <v>0.2750959834676621</v>
       </c>
       <c r="AK10" t="n">
-        <v>1.335883883545229</v>
+        <v>6.368300136054627</v>
       </c>
       <c r="AL10" t="n">
-        <v>28.98463816180137</v>
+        <v>66.05192839226406</v>
       </c>
       <c r="AM10" t="n">
         <v>9</v>
@@ -2060,10 +2060,10 @@
         <v>1.303547747924526</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.7211020829870098</v>
+        <v>5.866259378708966</v>
       </c>
       <c r="AR10" t="n">
-        <v>19.43506903835297</v>
+        <v>66.24446286353897</v>
       </c>
       <c r="AS10" t="n">
         <v>17</v>
@@ -2194,10 +2194,10 @@
         <v>0.3379617247761664</v>
       </c>
       <c r="AK11" t="n">
-        <v>1.18014588954017</v>
+        <v>6.212562142049567</v>
       </c>
       <c r="AL11" t="n">
-        <v>25.60559492317649</v>
+        <v>64.43661588999402</v>
       </c>
       <c r="AM11" t="n">
         <v>10</v>
@@ -2212,10 +2212,10 @@
         <v>0.957781661633594</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.699000304081913</v>
+        <v>5.844157599803869</v>
       </c>
       <c r="AR11" t="n">
-        <v>18.8393841706687</v>
+        <v>65.99487954691803</v>
       </c>
       <c r="AS11" t="n">
         <v>18</v>
@@ -2350,10 +2350,10 @@
         <v>0.4267180089400551</v>
       </c>
       <c r="AK12" t="n">
-        <v>1.137998416473196</v>
+        <v>6.170414668982594</v>
       </c>
       <c r="AL12" t="n">
-        <v>24.69112228724763</v>
+        <v>63.99946283290533</v>
       </c>
       <c r="AM12" t="n">
         <v>11</v>
@@ -2368,10 +2368,10 @@
         <v>-0.3545396137105352</v>
       </c>
       <c r="AQ12" t="n">
-        <v>1.642734172046797</v>
+        <v>6.787891467768752</v>
       </c>
       <c r="AR12" t="n">
-        <v>44.27480213778033</v>
+        <v>76.65195062638031</v>
       </c>
       <c r="AS12" t="n">
         <v>8</v>
@@ -2506,10 +2506,10 @@
         <v>0.3676249980257159</v>
       </c>
       <c r="AK13" t="n">
-        <v>1.083826895300926</v>
+        <v>6.116243147810324</v>
       </c>
       <c r="AL13" t="n">
-        <v>23.51576418974165</v>
+        <v>63.43759650108581</v>
       </c>
       <c r="AM13" t="n">
         <v>12</v>
@@ -2524,10 +2524,10 @@
         <v>0.3358942234891113</v>
       </c>
       <c r="AQ13" t="n">
-        <v>1.078201615207106</v>
+        <v>6.22335891092906</v>
       </c>
       <c r="AR13" t="n">
-        <v>29.05957883523583</v>
+        <v>70.27699282404463</v>
       </c>
       <c r="AS13" t="n">
         <v>9</v>
@@ -2656,10 +2656,10 @@
         <v>0.3643820871352654</v>
       </c>
       <c r="AK14" t="n">
-        <v>1.047744408653499</v>
+        <v>6.080160661162896</v>
       </c>
       <c r="AL14" t="n">
-        <v>22.73288340770974</v>
+        <v>63.06334940636152</v>
       </c>
       <c r="AM14" t="n">
         <v>13</v>
@@ -2674,10 +2674,10 @@
         <v>2.035742037550225</v>
       </c>
       <c r="AQ14" t="n">
-        <v>-0.2300855941668079</v>
+        <v>4.915071701555147</v>
       </c>
       <c r="AR14" t="n">
-        <v>-6.20124322597877</v>
+        <v>55.50321998836639</v>
       </c>
       <c r="AS14" t="n">
         <v>43</v>
@@ -2806,10 +2806,10 @@
         <v>0.3694008783697425</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.925920498023624</v>
+        <v>5.958336750533022</v>
       </c>
       <c r="AL15" t="n">
-        <v>20.08967316125348</v>
+        <v>61.79979334752676</v>
       </c>
       <c r="AM15" t="n">
         <v>14</v>
@@ -2824,10 +2824,10 @@
         <v>1.396032297803168</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0.05695475425542795</v>
+        <v>5.202112049977384</v>
       </c>
       <c r="AR15" t="n">
-        <v>1.535038668078026</v>
+        <v>58.74460985435265</v>
       </c>
       <c r="AS15" t="n">
         <v>32</v>
@@ -2966,10 +2966,10 @@
         <v>0.3714108204799814</v>
       </c>
       <c r="AK16" t="n">
-        <v>0.9208008323917458</v>
+        <v>5.953217084901143</v>
       </c>
       <c r="AL16" t="n">
-        <v>19.97859190810175</v>
+        <v>61.74669224040485</v>
       </c>
       <c r="AM16" t="n">
         <v>15</v>
@@ -2984,10 +2984,10 @@
         <v>0.2111304528617862</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.9823900623186027</v>
+        <v>6.127547358040558</v>
       </c>
       <c r="AR16" t="n">
-        <v>26.47727573420124</v>
+        <v>69.19504529198421</v>
       </c>
       <c r="AS16" t="n">
         <v>12</v>
@@ -3122,10 +3122,10 @@
         <v>0.304074617464679</v>
       </c>
       <c r="AK17" t="n">
-        <v>0.8706676472049013</v>
+        <v>5.903083899714298</v>
       </c>
       <c r="AL17" t="n">
-        <v>18.8908534823016</v>
+        <v>61.22671147830322</v>
       </c>
       <c r="AM17" t="n">
         <v>16</v>
@@ -3140,10 +3140,10 @@
         <v>0.02489835823143012</v>
       </c>
       <c r="AQ17" t="n">
-        <v>1.044238249772721</v>
+        <v>6.189395545494676</v>
       </c>
       <c r="AR17" t="n">
-        <v>28.14420170963133</v>
+        <v>69.89346308984899</v>
       </c>
       <c r="AS17" t="n">
         <v>10</v>
@@ -3274,10 +3274,10 @@
         <v>0.3726087901344018</v>
       </c>
       <c r="AK18" t="n">
-        <v>0.7953040326418599</v>
+        <v>5.827720285151258</v>
       </c>
       <c r="AL18" t="n">
-        <v>17.25569108115175</v>
+        <v>60.44504102211392</v>
       </c>
       <c r="AM18" t="n">
         <v>17</v>
@@ -3292,10 +3292,10 @@
         <v>-0.05708236093450922</v>
       </c>
       <c r="AQ18" t="n">
-        <v>1.008884501192515</v>
+        <v>6.154041796914471</v>
       </c>
       <c r="AR18" t="n">
-        <v>27.19135112074562</v>
+        <v>69.49423251825029</v>
       </c>
       <c r="AS18" t="n">
         <v>11</v>
@@ -3434,10 +3434,10 @@
         <v>0.3324440552156364</v>
       </c>
       <c r="AK19" t="n">
-        <v>0.7944670630644941</v>
+        <v>5.826883315573891</v>
       </c>
       <c r="AL19" t="n">
-        <v>17.23753137382149</v>
+        <v>60.43635998425302</v>
       </c>
       <c r="AM19" t="n">
         <v>18</v>
@@ -3452,10 +3452,10 @@
         <v>0.5764598348729143</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.5468410771422675</v>
+        <v>5.691998372864223</v>
       </c>
       <c r="AR19" t="n">
-        <v>14.73840436466847</v>
+        <v>64.27662851033217</v>
       </c>
       <c r="AS19" t="n">
         <v>22</v>
@@ -3586,10 +3586,10 @@
         <v>0.3577841699159819</v>
       </c>
       <c r="AK20" t="n">
-        <v>0.786314722930288</v>
+        <v>5.818730975439685</v>
       </c>
       <c r="AL20" t="n">
-        <v>17.0606502602214</v>
+        <v>60.3518040155848</v>
       </c>
       <c r="AM20" t="n">
         <v>19</v>
@@ -3604,10 +3604,10 @@
         <v>0.0434191818068049</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.9500631838010749</v>
+        <v>6.09522047952303</v>
       </c>
       <c r="AR20" t="n">
-        <v>25.60600503535634</v>
+        <v>68.82999551064984</v>
       </c>
       <c r="AS20" t="n">
         <v>13</v>
@@ -3738,10 +3738,10 @@
         <v>0.3826195348762376</v>
       </c>
       <c r="AK21" t="n">
-        <v>0.7574479243458817</v>
+        <v>5.789864176855279</v>
       </c>
       <c r="AL21" t="n">
-        <v>16.43432807596227</v>
+        <v>60.05239794610385</v>
       </c>
       <c r="AM21" t="n">
         <v>20</v>
@@ -3756,10 +3756,10 @@
         <v>1.047724630611241</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.2293936268211373</v>
+        <v>5.374550922543093</v>
       </c>
       <c r="AR21" t="n">
-        <v>6.182593393378527</v>
+        <v>60.6918678517349</v>
       </c>
       <c r="AS21" t="n">
         <v>28</v>
@@ -3890,10 +3890,10 @@
         <v>0.2852965317940014</v>
       </c>
       <c r="AK22" t="n">
-        <v>0.6104037820687207</v>
+        <v>5.642820034578119</v>
       </c>
       <c r="AL22" t="n">
-        <v>13.2439151140174</v>
+        <v>58.52725796389659</v>
       </c>
       <c r="AM22" t="n">
         <v>21</v>
@@ -3908,10 +3908,10 @@
         <v>0.6710184391178222</v>
       </c>
       <c r="AQ22" t="n">
-        <v>0.2752860704688032</v>
+        <v>5.420443366190759</v>
       </c>
       <c r="AR22" t="n">
-        <v>7.419481805815933</v>
+        <v>61.2101061502269</v>
       </c>
       <c r="AS22" t="n">
         <v>25</v>
@@ -4042,10 +4042,10 @@
         <v>0.3210273179535573</v>
       </c>
       <c r="AK23" t="n">
-        <v>0.5691454143530329</v>
+        <v>5.60156166686243</v>
       </c>
       <c r="AL23" t="n">
-        <v>12.34873337396067</v>
+        <v>58.09932669625589</v>
       </c>
       <c r="AM23" t="n">
         <v>22</v>
@@ -4060,10 +4060,10 @@
         <v>0.06126636961733242</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0.6560710470618734</v>
+        <v>5.80122834278383</v>
       </c>
       <c r="AR23" t="n">
-        <v>17.68235925889251</v>
+        <v>65.51010289644384</v>
       </c>
       <c r="AS23" t="n">
         <v>19</v>
@@ -4190,10 +4190,10 @@
         <v>0.2732232065447801</v>
       </c>
       <c r="AK24" t="n">
-        <v>0.5516669027826617</v>
+        <v>5.584083155292059</v>
       </c>
       <c r="AL24" t="n">
-        <v>11.96950255928118</v>
+        <v>57.91803979551556</v>
       </c>
       <c r="AM24" t="n">
         <v>23</v>
@@ -4208,10 +4208,10 @@
         <v>0.844026508249817</v>
       </c>
       <c r="AQ24" t="n">
-        <v>0.03374025436775474</v>
+        <v>5.178897550089711</v>
       </c>
       <c r="AR24" t="n">
-        <v>0.9093638591260547</v>
+        <v>58.48246118747201</v>
       </c>
       <c r="AS24" t="n">
         <v>33</v>
@@ -4342,10 +4342,10 @@
         <v>0.299279892116863</v>
       </c>
       <c r="AK25" t="n">
-        <v>0.5474062626997622</v>
+        <v>5.57982251520916</v>
       </c>
       <c r="AL25" t="n">
-        <v>11.87705956130685</v>
+        <v>57.8738484905129</v>
       </c>
       <c r="AM25" t="n">
         <v>24</v>
@@ -4360,10 +4360,10 @@
         <v>1.253698116981761</v>
       </c>
       <c r="AQ25" t="n">
-        <v>-0.2147696255591912</v>
+        <v>4.930387670162765</v>
       </c>
       <c r="AR25" t="n">
-        <v>-5.78844881822272</v>
+        <v>55.67617485588023</v>
       </c>
       <c r="AS25" t="n">
         <v>41</v>
@@ -4494,10 +4494,10 @@
         <v>0.2850741236300646</v>
       </c>
       <c r="AK26" t="n">
-        <v>0.5315704643215948</v>
+        <v>5.563986716830992</v>
       </c>
       <c r="AL26" t="n">
-        <v>11.53347065238437</v>
+        <v>57.70959979020635</v>
       </c>
       <c r="AM26" t="n">
         <v>25</v>
@@ -4512,10 +4512,10 @@
         <v>1.068414777751088</v>
       </c>
       <c r="AQ26" t="n">
-        <v>-0.1925482540413546</v>
+        <v>4.952609041680601</v>
       </c>
       <c r="AR26" t="n">
-        <v>-5.1895407027627</v>
+        <v>55.9271086665523</v>
       </c>
       <c r="AS26" t="n">
         <v>38</v>
@@ -4646,10 +4646,10 @@
         <v>0.2845895009129479</v>
       </c>
       <c r="AK27" t="n">
-        <v>0.4825378005580863</v>
+        <v>5.514954053067484</v>
       </c>
       <c r="AL27" t="n">
-        <v>10.46961021151811</v>
+        <v>57.20103362237561</v>
       </c>
       <c r="AM27" t="n">
         <v>26</v>
@@ -4664,10 +4664,10 @@
         <v>0.8978605473667873</v>
       </c>
       <c r="AQ27" t="n">
-        <v>-0.08635408753821955</v>
+        <v>5.058803208183736</v>
       </c>
       <c r="AR27" t="n">
-        <v>-2.327406469410387</v>
+        <v>57.12630138291487</v>
       </c>
       <c r="AS27" t="n">
         <v>37</v>
@@ -4802,10 +4802,10 @@
         <v>0.3250293286571209</v>
       </c>
       <c r="AK28" t="n">
-        <v>0.4462650849477238</v>
+        <v>5.478681337457121</v>
       </c>
       <c r="AL28" t="n">
-        <v>9.682602036584404</v>
+        <v>56.82481347525594</v>
       </c>
       <c r="AM28" t="n">
         <v>27</v>
@@ -4820,10 +4820,10 @@
         <v>-0.3545396137105352</v>
       </c>
       <c r="AQ28" t="n">
-        <v>0.7703999055856054</v>
+        <v>5.915557201307561</v>
       </c>
       <c r="AR28" t="n">
-        <v>20.7637388733858</v>
+        <v>66.80115624641914</v>
       </c>
       <c r="AS28" t="n">
         <v>16</v>
@@ -4954,10 +4954,10 @@
         <v>0.2790217494123259</v>
       </c>
       <c r="AK29" t="n">
-        <v>0.4132535559406129</v>
+        <v>5.44566980845001</v>
       </c>
       <c r="AL29" t="n">
-        <v>8.966351743258276</v>
+        <v>56.48241831430053</v>
       </c>
       <c r="AM29" t="n">
         <v>28</v>
@@ -4972,10 +4972,10 @@
         <v>0.2830751662802494</v>
       </c>
       <c r="AQ29" t="n">
-        <v>0.2424875915158327</v>
+        <v>5.387644887237788</v>
       </c>
       <c r="AR29" t="n">
-        <v>6.535500580628664</v>
+        <v>60.83973084277521</v>
       </c>
       <c r="AS29" t="n">
         <v>26</v>
@@ -5100,10 +5100,10 @@
         <v>0.3865650960335092</v>
       </c>
       <c r="AK30" t="n">
-        <v>0.3651793268440849</v>
+        <v>5.397595579353482</v>
       </c>
       <c r="AL30" t="n">
-        <v>7.923286434638413</v>
+        <v>55.98379301870251</v>
       </c>
       <c r="AM30" t="n">
         <v>29</v>
@@ -5118,10 +5118,10 @@
         <v>1.860033694410872</v>
       </c>
       <c r="AQ30" t="n">
-        <v>-0.8821120106475893</v>
+        <v>4.263045285074367</v>
       </c>
       <c r="AR30" t="n">
-        <v>-23.77459201820817</v>
+        <v>48.14024182047751</v>
       </c>
       <c r="AS30" t="n">
         <v>59</v>
@@ -5246,10 +5246,10 @@
         <v>0.3970547356905056</v>
       </c>
       <c r="AK31" t="n">
-        <v>0.3546102557822872</v>
+        <v>5.387026508291685</v>
       </c>
       <c r="AL31" t="n">
-        <v>7.693969572442581</v>
+        <v>55.87417074744771</v>
       </c>
       <c r="AM31" t="n">
         <v>30</v>
@@ -5264,10 +5264,10 @@
         <v>0.4592251651346725</v>
       </c>
       <c r="AQ31" t="n">
-        <v>-0.003035147698903284</v>
+        <v>5.142122148023052</v>
       </c>
       <c r="AR31" t="n">
-        <v>-0.08180298803941484</v>
+        <v>58.06717665959411</v>
       </c>
       <c r="AS31" t="n">
         <v>34</v>
@@ -5394,10 +5394,10 @@
         <v>0.3194675331802836</v>
       </c>
       <c r="AK32" t="n">
-        <v>0.2970413102882732</v>
+        <v>5.329457562797671</v>
       </c>
       <c r="AL32" t="n">
-        <v>6.444897647065195</v>
+        <v>55.27706637357243</v>
       </c>
       <c r="AM32" t="n">
         <v>31</v>
@@ -5412,10 +5412,10 @@
         <v>0.7545533751889902</v>
       </c>
       <c r="AQ32" t="n">
-        <v>-0.19722329403084</v>
+        <v>4.947934001691116</v>
       </c>
       <c r="AR32" t="n">
-        <v>-5.315541898843485</v>
+        <v>55.8743159935769</v>
       </c>
       <c r="AS32" t="n">
         <v>39</v>
@@ -5546,10 +5546,10 @@
         <v>0.2901996427125294</v>
       </c>
       <c r="AK33" t="n">
-        <v>0.2445590671742046</v>
+        <v>5.276975319683602</v>
       </c>
       <c r="AL33" t="n">
-        <v>5.306191772012643</v>
+        <v>54.73272121238732</v>
       </c>
       <c r="AM33" t="n">
         <v>32</v>
@@ -5564,10 +5564,10 @@
         <v>0.06126636961733242</v>
       </c>
       <c r="AQ33" t="n">
-        <v>0.236082280291586</v>
+        <v>5.381239576013542</v>
       </c>
       <c r="AR33" t="n">
-        <v>6.362865292515631</v>
+        <v>60.76739916186386</v>
       </c>
       <c r="AS33" t="n">
         <v>27</v>
@@ -5702,10 +5702,10 @@
         <v>0.2648040516901551</v>
       </c>
       <c r="AK34" t="n">
-        <v>0.225766275899532</v>
+        <v>5.25818252840893</v>
       </c>
       <c r="AL34" t="n">
-        <v>4.898445064491115</v>
+        <v>54.53780261919196</v>
       </c>
       <c r="AM34" t="n">
         <v>33</v>
@@ -5720,10 +5720,10 @@
         <v>0.2717932078585836</v>
       </c>
       <c r="AQ34" t="n">
-        <v>0.06123662824286401</v>
+        <v>5.20639392396482</v>
       </c>
       <c r="AR34" t="n">
-        <v>1.650443294583379</v>
+        <v>58.79296271842419</v>
       </c>
       <c r="AS34" t="n">
         <v>31</v>
@@ -5854,10 +5854,10 @@
         <v>0.3263188805831577</v>
       </c>
       <c r="AK35" t="n">
-        <v>0.2012339185510105</v>
+        <v>5.233650171060408</v>
       </c>
       <c r="AL35" t="n">
-        <v>4.366167139918914</v>
+        <v>54.28335331933817</v>
       </c>
       <c r="AM35" t="n">
         <v>34</v>
@@ -5872,10 +5872,10 @@
         <v>0.1980431818794646</v>
       </c>
       <c r="AQ35" t="n">
-        <v>0.08370836617501892</v>
+        <v>5.228865661896974</v>
       </c>
       <c r="AR35" t="n">
-        <v>2.256099259844366</v>
+        <v>59.04672378025663</v>
       </c>
       <c r="AS35" t="n">
         <v>30</v>
@@ -6006,10 +6006,10 @@
         <v>0.3665831421999937</v>
       </c>
       <c r="AK36" t="n">
-        <v>0.1500202801982075</v>
+        <v>5.182436532707604</v>
       </c>
       <c r="AL36" t="n">
-        <v>3.254986149647547</v>
+        <v>53.75216611067711</v>
       </c>
       <c r="AM36" t="n">
         <v>35</v>
@@ -6024,10 +6024,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ36" t="n">
-        <v>0.5080680276774867</v>
+        <v>5.653225323399442</v>
       </c>
       <c r="AR36" t="n">
-        <v>13.69339713066626</v>
+        <v>63.83878564155315</v>
       </c>
       <c r="AS36" t="n">
         <v>23</v>
@@ -6162,10 +6162,10 @@
         <v>0.4040667337925105</v>
       </c>
       <c r="AK37" t="n">
-        <v>0.002391754174868255</v>
+        <v>5.034808006684266</v>
       </c>
       <c r="AL37" t="n">
-        <v>0.05189382863618253</v>
+        <v>52.22096490765244</v>
       </c>
       <c r="AM37" t="n">
         <v>36</v>
@@ -6180,10 +6180,10 @@
         <v>-1.233834065898723</v>
       </c>
       <c r="AQ37" t="n">
-        <v>0.9237787914828566</v>
+        <v>6.068936087204812</v>
       </c>
       <c r="AR37" t="n">
-        <v>24.89759080193784</v>
+        <v>68.53318022540445</v>
       </c>
       <c r="AS37" t="n">
         <v>14</v>
@@ -6314,10 +6314,10 @@
         <v>0.3263188805831577</v>
       </c>
       <c r="AK38" t="n">
-        <v>-0.01971183442074065</v>
+        <v>5.012704418088656</v>
       </c>
       <c r="AL38" t="n">
-        <v>-0.4276871629548071</v>
+        <v>51.99170676655707</v>
       </c>
       <c r="AM38" t="n">
         <v>37</v>
@@ -6332,10 +6332,10 @@
         <v>-0.694697140925294</v>
       </c>
       <c r="AQ38" t="n">
-        <v>0.4423972742405439</v>
+        <v>5.5875545699625</v>
       </c>
       <c r="AR38" t="n">
-        <v>11.92344575074405</v>
+        <v>63.0972016940272</v>
       </c>
       <c r="AS38" t="n">
         <v>24</v>
@@ -6462,10 +6462,10 @@
         <v>0.2922524259931254</v>
       </c>
       <c r="AK39" t="n">
-        <v>-0.1095796797408947</v>
+        <v>4.922836572768503</v>
       </c>
       <c r="AL39" t="n">
-        <v>-2.377547484701257</v>
+        <v>51.05959861256994</v>
       </c>
       <c r="AM39" t="n">
         <v>38</v>
@@ -6480,10 +6480,10 @@
         <v>-0.01438208649577635</v>
       </c>
       <c r="AQ39" t="n">
-        <v>-0.06071402072592497</v>
+        <v>5.084443274996031</v>
       </c>
       <c r="AR39" t="n">
-        <v>-1.636358030636283</v>
+        <v>57.41584065216885</v>
       </c>
       <c r="AS39" t="n">
         <v>36</v>
@@ -6614,10 +6614,10 @@
         <v>0.3539571725515125</v>
       </c>
       <c r="AK40" t="n">
-        <v>-0.1453280962460377</v>
+        <v>4.88708815626336</v>
       </c>
       <c r="AL40" t="n">
-        <v>-3.15317995547345</v>
+        <v>50.6888164891323</v>
       </c>
       <c r="AM40" t="n">
         <v>39</v>
@@ -6632,10 +6632,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ40" t="n">
-        <v>0.5877877780666269</v>
+        <v>5.732945073788582</v>
       </c>
       <c r="AR40" t="n">
-        <v>15.84199562883634</v>
+        <v>64.73901723774047</v>
       </c>
       <c r="AS40" t="n">
         <v>21</v>
@@ -6766,10 +6766,10 @@
         <v>0.2806966026870421</v>
       </c>
       <c r="AK41" t="n">
-        <v>-0.1718096623596011</v>
+        <v>4.860606590149796</v>
       </c>
       <c r="AL41" t="n">
-        <v>-3.727749812340407</v>
+        <v>50.41415002064331</v>
       </c>
       <c r="AM41" t="n">
         <v>40</v>
@@ -6784,10 +6784,10 @@
         <v>-0.03526794393837076</v>
       </c>
       <c r="AQ41" t="n">
-        <v>-0.2059128758320017</v>
+        <v>4.939244419889954</v>
       </c>
       <c r="AR41" t="n">
-        <v>-5.549742612174437</v>
+        <v>55.7761892927672</v>
       </c>
       <c r="AS41" t="n">
         <v>40</v>
@@ -6922,10 +6922,10 @@
         <v>0.3401045896210866</v>
       </c>
       <c r="AK42" t="n">
-        <v>-0.1745660669806209</v>
+        <v>4.857850185528776</v>
       </c>
       <c r="AL42" t="n">
-        <v>-3.787555452300484</v>
+        <v>50.38556062680853</v>
       </c>
       <c r="AM42" t="n">
         <v>41</v>
@@ -6940,10 +6940,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ42" t="n">
-        <v>0.08807926090719936</v>
+        <v>5.233236556629155</v>
       </c>
       <c r="AR42" t="n">
-        <v>2.373903164289377</v>
+        <v>59.09608190697317</v>
       </c>
       <c r="AS42" t="n">
         <v>29</v>
@@ -7074,10 +7074,10 @@
         <v>0.3356551602420135</v>
       </c>
       <c r="AK43" t="n">
-        <v>-0.2248186888503115</v>
+        <v>4.807597563659086</v>
       </c>
       <c r="AL43" t="n">
-        <v>-4.877885292727437</v>
+        <v>49.86434106894443</v>
       </c>
       <c r="AM43" t="n">
         <v>42</v>
@@ -7092,10 +7092,10 @@
         <v>-1.233834065898723</v>
       </c>
       <c r="AQ43" t="n">
-        <v>0.6297866547436555</v>
+        <v>5.774943950465611</v>
       </c>
       <c r="AR43" t="n">
-        <v>16.97394502547402</v>
+        <v>65.21328761119845</v>
       </c>
       <c r="AS43" t="n">
         <v>20</v>
@@ -7226,10 +7226,10 @@
         <v>0.221365545492914</v>
       </c>
       <c r="AK44" t="n">
-        <v>-0.2529918948184983</v>
+        <v>4.779424357690899</v>
       </c>
       <c r="AL44" t="n">
-        <v>-5.489158615883856</v>
+        <v>49.57212893329843</v>
       </c>
       <c r="AM44" t="n">
         <v>43</v>
@@ -7244,10 +7244,10 @@
         <v>-0.01438208649577635</v>
       </c>
       <c r="AQ44" t="n">
-        <v>-0.3389097374532916</v>
+        <v>4.806247558268664</v>
       </c>
       <c r="AR44" t="n">
-        <v>-9.134260322603252</v>
+        <v>54.27432838074974</v>
       </c>
       <c r="AS44" t="n">
         <v>44</v>
@@ -7382,10 +7382,10 @@
         <v>0.2235554316005274</v>
       </c>
       <c r="AK45" t="n">
-        <v>-0.2652385392935504</v>
+        <v>4.767177713215847</v>
       </c>
       <c r="AL45" t="n">
-        <v>-5.754873745153617</v>
+        <v>49.44510689183844</v>
       </c>
       <c r="AM45" t="n">
         <v>44</v>
@@ -7400,10 +7400,10 @@
         <v>0.4014238968320915</v>
       </c>
       <c r="AQ45" t="n">
-        <v>-0.5905685485970144</v>
+        <v>4.554588747124941</v>
       </c>
       <c r="AR45" t="n">
-        <v>-15.91694266964092</v>
+        <v>51.4324828889533</v>
       </c>
       <c r="AS45" t="n">
         <v>51</v>
@@ -7534,10 +7534,10 @@
         <v>0.2065885180129795</v>
       </c>
       <c r="AK46" t="n">
-        <v>-0.2894802551476546</v>
+        <v>4.742935997361743</v>
       </c>
       <c r="AL46" t="n">
-        <v>-6.280845628718619</v>
+        <v>49.19367212188538</v>
       </c>
       <c r="AM46" t="n">
         <v>45</v>
@@ -7552,10 +7552,10 @@
         <v>0.06126636961733242</v>
       </c>
       <c r="AQ46" t="n">
-        <v>-0.4200638528493508</v>
+        <v>4.725093442872605</v>
       </c>
       <c r="AR46" t="n">
-        <v>-11.32151767864294</v>
+        <v>53.35789928402596</v>
       </c>
       <c r="AS46" t="n">
         <v>46</v>
@@ -7686,10 +7686,10 @@
         <v>0.3149126893168235</v>
       </c>
       <c r="AK47" t="n">
-        <v>-0.2978903700514551</v>
+        <v>4.734525882457942</v>
       </c>
       <c r="AL47" t="n">
-        <v>-6.463319674845232</v>
+        <v>49.10644251657021</v>
       </c>
       <c r="AM47" t="n">
         <v>46</v>
@@ -7704,10 +7704,10 @@
         <v>-0.4957177431666238</v>
       </c>
       <c r="AQ47" t="n">
-        <v>-0.003877461319532954</v>
+        <v>5.141279834402423</v>
       </c>
       <c r="AR47" t="n">
-        <v>-0.1045049379506836</v>
+        <v>58.05766487196949</v>
       </c>
       <c r="AS47" t="n">
         <v>35</v>
@@ -7838,10 +7838,10 @@
         <v>0.2580868334324917</v>
       </c>
       <c r="AK48" t="n">
-        <v>-0.3009561782582524</v>
+        <v>4.731460074251145</v>
       </c>
       <c r="AL48" t="n">
-        <v>-6.529838436424774</v>
+        <v>49.07464399266063</v>
       </c>
       <c r="AM48" t="n">
         <v>47</v>
@@ -7856,10 +7856,10 @@
         <v>0.1267960429603123</v>
       </c>
       <c r="AQ48" t="n">
-        <v>-0.4588503651089607</v>
+        <v>4.686306930612995</v>
       </c>
       <c r="AR48" t="n">
-        <v>-12.36688776050418</v>
+        <v>52.91990438725865</v>
       </c>
       <c r="AS48" t="n">
         <v>47</v>
@@ -7986,10 +7986,10 @@
         <v>0.1990824080032964</v>
       </c>
       <c r="AK49" t="n">
-        <v>-0.4014988052908441</v>
+        <v>4.630917447218553</v>
       </c>
       <c r="AL49" t="n">
-        <v>-8.711309221627156</v>
+        <v>48.03181713788848</v>
       </c>
       <c r="AM49" t="n">
         <v>48</v>
@@ -8004,10 +8004,10 @@
         <v>-0.1836103404515539</v>
       </c>
       <c r="AQ49" t="n">
-        <v>-0.392917056861246</v>
+        <v>4.752240238860709</v>
       </c>
       <c r="AR49" t="n">
-        <v>-10.58986003037567</v>
+        <v>53.66445322284854</v>
       </c>
       <c r="AS49" t="n">
         <v>45</v>
@@ -8134,10 +8134,10 @@
         <v>0.3174526333322049</v>
       </c>
       <c r="AK50" t="n">
-        <v>-0.4392404101822858</v>
+        <v>4.593175842327112</v>
       </c>
       <c r="AL50" t="n">
-        <v>-9.530187849402049</v>
+        <v>47.64036168974074</v>
       </c>
       <c r="AM50" t="n">
         <v>49</v>
@@ -8152,10 +8152,10 @@
         <v>0.1565471867632049</v>
       </c>
       <c r="AQ50" t="n">
-        <v>-0.6127273562567743</v>
+        <v>4.532429939465182</v>
       </c>
       <c r="AR50" t="n">
-        <v>-16.51416457044464</v>
+        <v>51.18225557775651</v>
       </c>
       <c r="AS50" t="n">
         <v>52</v>
@@ -8280,10 +8280,10 @@
         <v>0.2870981812969297</v>
       </c>
       <c r="AK51" t="n">
-        <v>-0.5002940449787388</v>
+        <v>4.532122207530659</v>
       </c>
       <c r="AL51" t="n">
-        <v>-10.85486698868597</v>
+        <v>47.00711416253466</v>
       </c>
       <c r="AM51" t="n">
         <v>50</v>
@@ -8298,10 +8298,10 @@
         <v>0.4014238968320915</v>
       </c>
       <c r="AQ51" t="n">
-        <v>-0.9849604554538706</v>
+        <v>4.160196840268085</v>
       </c>
       <c r="AR51" t="n">
-        <v>-26.54655270512983</v>
+        <v>46.97883051171914</v>
       </c>
       <c r="AS51" t="n">
         <v>65</v>
@@ -8426,10 +8426,10 @@
         <v>0.3118590083829335</v>
       </c>
       <c r="AK52" t="n">
-        <v>-0.5031082087843415</v>
+        <v>4.529308043725056</v>
       </c>
       <c r="AL52" t="n">
-        <v>-10.91592582818403</v>
+        <v>46.97792569116858</v>
       </c>
       <c r="AM52" t="n">
         <v>51</v>
@@ -8444,10 +8444,10 @@
         <v>0.2363023076581557</v>
       </c>
       <c r="AQ52" t="n">
-        <v>-0.8911351411592157</v>
+        <v>4.254022154562739</v>
       </c>
       <c r="AR52" t="n">
-        <v>-24.01778250201473</v>
+        <v>48.03834853627331</v>
       </c>
       <c r="AS52" t="n">
         <v>60</v>
@@ -8572,10 +8572,10 @@
         <v>0.3440278126689904</v>
       </c>
       <c r="AK53" t="n">
-        <v>-0.51388558712985</v>
+        <v>4.518530665379547</v>
       </c>
       <c r="AL53" t="n">
-        <v>-11.14976232814119</v>
+        <v>46.86614285940417</v>
       </c>
       <c r="AM53" t="n">
         <v>52</v>
@@ -8590,10 +8590,10 @@
         <v>0.2717932078585836</v>
       </c>
       <c r="AQ53" t="n">
-        <v>-0.9145430197212725</v>
+        <v>4.230614276000683</v>
       </c>
       <c r="AR53" t="n">
-        <v>-24.64866923307296</v>
+        <v>47.77401614965121</v>
       </c>
       <c r="AS53" t="n">
         <v>61</v>
@@ -8724,10 +8724,10 @@
         <v>0.2814732852646757</v>
       </c>
       <c r="AK54" t="n">
-        <v>-0.6191531662547903</v>
+        <v>4.413263086254608</v>
       </c>
       <c r="AL54" t="n">
-        <v>-13.43375027700987</v>
+        <v>45.77430886134528</v>
       </c>
       <c r="AM54" t="n">
         <v>53</v>
@@ -8742,10 +8742,10 @@
         <v>-0.2133614842544465</v>
       </c>
       <c r="AQ54" t="n">
-        <v>-0.5856953289592697</v>
+        <v>4.559461966762686</v>
       </c>
       <c r="AR54" t="n">
-        <v>-15.78560015610067</v>
+        <v>51.48751349644571</v>
       </c>
       <c r="AS54" t="n">
         <v>50</v>
@@ -8876,10 +8876,10 @@
         <v>0.253101602976853</v>
       </c>
       <c r="AK55" t="n">
-        <v>-0.6601756008112291</v>
+        <v>4.372240651698169</v>
       </c>
       <c r="AL55" t="n">
-        <v>-14.32381298139633</v>
+        <v>45.34882468944554</v>
       </c>
       <c r="AM55" t="n">
         <v>54</v>
@@ -8894,10 +8894,10 @@
         <v>-0.7841702739861206</v>
       </c>
       <c r="AQ55" t="n">
-        <v>-0.2214427315859177</v>
+        <v>4.923714564136038</v>
       </c>
       <c r="AR55" t="n">
-        <v>-5.968301684258628</v>
+        <v>55.6008191145408</v>
       </c>
       <c r="AS55" t="n">
         <v>42</v>
@@ -9028,10 +9028,10 @@
         <v>0.2746344269206095</v>
       </c>
       <c r="AK56" t="n">
-        <v>-0.6840042593254062</v>
+        <v>4.348411993183992</v>
       </c>
       <c r="AL56" t="n">
-        <v>-14.84082277051185</v>
+        <v>45.10167414499314</v>
       </c>
       <c r="AM56" t="n">
         <v>55</v>
@@ -9046,10 +9046,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ56" t="n">
-        <v>-0.5016975756052122</v>
+        <v>4.643459720116743</v>
       </c>
       <c r="AR56" t="n">
-        <v>-13.52170136282529</v>
+        <v>52.4360542433617</v>
       </c>
       <c r="AS56" t="n">
         <v>49</v>
@@ -9180,10 +9180,10 @@
         <v>0.2708082613128754</v>
       </c>
       <c r="AK57" t="n">
-        <v>-0.7949371996516397</v>
+        <v>4.237479052857758</v>
       </c>
       <c r="AL57" t="n">
-        <v>-17.24773191522549</v>
+        <v>43.95107909227453</v>
       </c>
       <c r="AM57" t="n">
         <v>56</v>
@@ -9198,10 +9198,10 @@
         <v>-0.694697140925294</v>
       </c>
       <c r="AQ57" t="n">
-        <v>-0.4785396783065924</v>
+        <v>4.666617617415364</v>
       </c>
       <c r="AR57" t="n">
-        <v>-12.89755210102116</v>
+        <v>52.69756372812195</v>
       </c>
       <c r="AS57" t="n">
         <v>48</v>
@@ -9328,10 +9328,10 @@
         <v>0.2072860263138315</v>
       </c>
       <c r="AK58" t="n">
-        <v>-0.8162114715714535</v>
+        <v>4.216204780937944</v>
       </c>
       <c r="AL58" t="n">
-        <v>-17.7093192442942</v>
+        <v>43.73042261324186</v>
       </c>
       <c r="AM58" t="n">
         <v>57</v>
@@ -9346,10 +9346,10 @@
         <v>-0.1290270743529726</v>
       </c>
       <c r="AQ58" t="n">
-        <v>-0.9210085953571566</v>
+        <v>4.224148700364799</v>
       </c>
       <c r="AR58" t="n">
-        <v>-24.82292876139881</v>
+        <v>47.70100393565719</v>
       </c>
       <c r="AS58" t="n">
         <v>63</v>
@@ -9476,10 +9476,10 @@
         <v>0.2945287128778097</v>
       </c>
       <c r="AK59" t="n">
-        <v>-0.8393543036732253</v>
+        <v>4.193061948836172</v>
       </c>
       <c r="AL59" t="n">
-        <v>-18.21144867543084</v>
+        <v>43.49038545165678</v>
       </c>
       <c r="AM59" t="n">
         <v>58</v>
@@ -9494,10 +9494,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ59" t="n">
-        <v>-0.7154782782879485</v>
+        <v>4.429679017434007</v>
       </c>
       <c r="AR59" t="n">
-        <v>-19.28349683358035</v>
+        <v>50.021945540428</v>
       </c>
       <c r="AS59" t="n">
         <v>55</v>
@@ -9624,10 +9624,10 @@
         <v>0.2135455274391398</v>
       </c>
       <c r="AK60" t="n">
-        <v>-0.8403657079989424</v>
+        <v>4.192050544510455</v>
       </c>
       <c r="AL60" t="n">
-        <v>-18.23339308899648</v>
+        <v>43.47989517879422</v>
       </c>
       <c r="AM60" t="n">
         <v>59</v>
@@ -9642,10 +9642,10 @@
         <v>-0.1555602159518652</v>
       </c>
       <c r="AQ60" t="n">
-        <v>-0.919729988853504</v>
+        <v>4.225427306868451</v>
       </c>
       <c r="AR60" t="n">
-        <v>-24.78846789065989</v>
+        <v>47.71544254049552</v>
       </c>
       <c r="AS60" t="n">
         <v>62</v>
@@ -9772,10 +9772,10 @@
         <v>0.2376569080368338</v>
       </c>
       <c r="AK61" t="n">
-        <v>-0.9061581402993673</v>
+        <v>4.126258112210031</v>
       </c>
       <c r="AL61" t="n">
-        <v>-19.66088979548554</v>
+        <v>42.79749690386731</v>
       </c>
       <c r="AM61" t="n">
         <v>60</v>
@@ -9790,10 +9790,10 @@
         <v>0.1418970368241607</v>
       </c>
       <c r="AQ61" t="n">
-        <v>-1.215678479114701</v>
+        <v>3.929478816607255</v>
       </c>
       <c r="AR61" t="n">
-        <v>-32.76484110566599</v>
+        <v>44.37345789457574</v>
       </c>
       <c r="AS61" t="n">
         <v>73</v>
@@ -9918,10 +9918,10 @@
         <v>0.2351407784406057</v>
       </c>
       <c r="AK62" t="n">
-        <v>-0.9067428641223751</v>
+        <v>4.125673388387022</v>
       </c>
       <c r="AL62" t="n">
-        <v>-19.67357653319024</v>
+        <v>42.79143215577731</v>
       </c>
       <c r="AM62" t="n">
         <v>61</v>
@@ -9936,10 +9936,10 @@
         <v>0.3257754407189825</v>
       </c>
       <c r="AQ62" t="n">
-        <v>-1.434226918401224</v>
+        <v>3.710930377320731</v>
       </c>
       <c r="AR62" t="n">
-        <v>-38.65513612209904</v>
+        <v>41.90550974643458</v>
       </c>
       <c r="AS62" t="n">
         <v>78</v>
@@ -10064,10 +10064,10 @@
         <v>0.3044649423397373</v>
       </c>
       <c r="AK63" t="n">
-        <v>-0.9453191367887563</v>
+        <v>4.087097115720641</v>
       </c>
       <c r="AL63" t="n">
-        <v>-20.51056492614752</v>
+        <v>42.3913195440343</v>
       </c>
       <c r="AM63" t="n">
         <v>62</v>
@@ -10082,10 +10082,10 @@
         <v>-0.2133614842544465</v>
       </c>
       <c r="AQ63" t="n">
-        <v>-1.090285909600666</v>
+        <v>4.05487138612129</v>
       </c>
       <c r="AR63" t="n">
-        <v>-29.38527349256614</v>
+        <v>45.78944768948391</v>
       </c>
       <c r="AS63" t="n">
         <v>68</v>
@@ -10210,10 +10210,10 @@
         <v>0.2256377384151184</v>
       </c>
       <c r="AK64" t="n">
-        <v>-0.9479455451839672</v>
+        <v>4.08447070732543</v>
       </c>
       <c r="AL64" t="n">
-        <v>-20.5675500413495</v>
+        <v>42.36407846940794</v>
       </c>
       <c r="AM64" t="n">
         <v>63</v>
@@ -10228,10 +10228,10 @@
         <v>0.7099095592886046</v>
       </c>
       <c r="AQ64" t="n">
-        <v>-1.735906356670843</v>
+        <v>3.409250939051113</v>
       </c>
       <c r="AR64" t="n">
-        <v>-46.78596925731162</v>
+        <v>38.49880863504539</v>
       </c>
       <c r="AS64" t="n">
         <v>88</v>
@@ -10358,10 +10358,10 @@
         <v>0.2450030567271742</v>
       </c>
       <c r="AK65" t="n">
-        <v>-1.001789701440126</v>
+        <v>4.030626551069272</v>
       </c>
       <c r="AL65" t="n">
-        <v>-21.73580531071507</v>
+        <v>41.80560756235408</v>
       </c>
       <c r="AM65" t="n">
         <v>64</v>
@@ -10376,10 +10376,10 @@
         <v>-0.6190486848121851</v>
       </c>
       <c r="AQ65" t="n">
-        <v>-0.7436718754408971</v>
+        <v>4.401485420281058</v>
       </c>
       <c r="AR65" t="n">
-        <v>-20.04336775898016</v>
+        <v>49.70357064784029</v>
       </c>
       <c r="AS65" t="n">
         <v>56</v>
@@ -10506,10 +10506,10 @@
         <v>0.3115437796443196</v>
       </c>
       <c r="AK66" t="n">
-        <v>-1.018630596766642</v>
+        <v>4.013785655742755</v>
       </c>
       <c r="AL66" t="n">
-        <v>-22.10120178219913</v>
+        <v>41.63093400922317</v>
       </c>
       <c r="AM66" t="n">
         <v>65</v>
@@ -10524,10 +10524,10 @@
         <v>-0.7841702739861206</v>
       </c>
       <c r="AQ66" t="n">
-        <v>-0.7090654904941819</v>
+        <v>4.436091805227774</v>
       </c>
       <c r="AR66" t="n">
-        <v>-19.110660037736</v>
+        <v>50.09436165015505</v>
       </c>
       <c r="AS66" t="n">
         <v>54</v>
@@ -10654,10 +10654,10 @@
         <v>0.1966047184069102</v>
       </c>
       <c r="AK67" t="n">
-        <v>-1.032072248020337</v>
+        <v>4.00034400448906</v>
       </c>
       <c r="AL67" t="n">
-        <v>-22.39284494271958</v>
+        <v>41.49151737258316</v>
       </c>
       <c r="AM67" t="n">
         <v>66</v>
@@ -10672,10 +10672,10 @@
         <v>-0.6190486848121851</v>
       </c>
       <c r="AQ67" t="n">
-        <v>-0.8773761992477257</v>
+        <v>4.267781096474231</v>
       </c>
       <c r="AR67" t="n">
-        <v>-23.64695291733675</v>
+        <v>48.19372075179542</v>
       </c>
       <c r="AS67" t="n">
         <v>58</v>
@@ -10802,10 +10802,10 @@
         <v>0.2635940522233673</v>
       </c>
       <c r="AK68" t="n">
-        <v>-1.098068108776324</v>
+        <v>3.934348143733073</v>
       </c>
       <c r="AL68" t="n">
-        <v>-23.82475543116147</v>
+        <v>40.80700914029044</v>
       </c>
       <c r="AM68" t="n">
         <v>67</v>
@@ -10820,10 +10820,10 @@
         <v>-0.1555602159518652</v>
       </c>
       <c r="AQ68" t="n">
-        <v>-1.205659518888213</v>
+        <v>3.939497776833742</v>
       </c>
       <c r="AR68" t="n">
-        <v>-32.49481112199473</v>
+        <v>44.48659653980232</v>
       </c>
       <c r="AS68" t="n">
         <v>72</v>
@@ -10950,10 +10950,10 @@
         <v>0.2456642359801274</v>
       </c>
       <c r="AK69" t="n">
-        <v>-1.101863639129026</v>
+        <v>3.930552613380372</v>
       </c>
       <c r="AL69" t="n">
-        <v>-23.90710695531733</v>
+        <v>40.76764194752138</v>
       </c>
       <c r="AM69" t="n">
         <v>68</v>
@@ -10968,10 +10968,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ69" t="n">
-        <v>-0.6459410187134778</v>
+        <v>4.499216277008478</v>
       </c>
       <c r="AR69" t="n">
-        <v>-17.40933577864403</v>
+        <v>50.80719182978098</v>
       </c>
       <c r="AS69" t="n">
         <v>53</v>
@@ -11098,10 +11098,10 @@
         <v>0.2069206286229998</v>
       </c>
       <c r="AK70" t="n">
-        <v>-1.174136719090389</v>
+        <v>3.858279533419009</v>
       </c>
       <c r="AL70" t="n">
-        <v>-25.47521410693574</v>
+        <v>40.01802647709636</v>
       </c>
       <c r="AM70" t="n">
         <v>69</v>
@@ -11116,10 +11116,10 @@
         <v>0.1707726343151758</v>
       </c>
       <c r="AQ70" t="n">
-        <v>-1.541650532304443</v>
+        <v>3.603506763417513</v>
       </c>
       <c r="AR70" t="n">
-        <v>-41.55040629509623</v>
+        <v>40.69243355213833</v>
       </c>
       <c r="AS70" t="n">
         <v>81</v>
@@ -11244,10 +11244,10 @@
         <v>0.2988983082795889</v>
       </c>
       <c r="AK71" t="n">
-        <v>-1.280592576511043</v>
+        <v>3.751823675998354</v>
       </c>
       <c r="AL71" t="n">
-        <v>-27.78498409933457</v>
+        <v>38.9138676715972</v>
       </c>
       <c r="AM71" t="n">
         <v>70</v>
@@ -11262,10 +11262,10 @@
         <v>-0.2788911575974264</v>
       </c>
       <c r="AQ71" t="n">
-        <v>-1.436023457002074</v>
+        <v>3.709133838719882</v>
       </c>
       <c r="AR71" t="n">
-        <v>-38.70355624535392</v>
+        <v>41.88522241733031</v>
       </c>
       <c r="AS71" t="n">
         <v>79</v>
@@ -11392,10 +11392,10 @@
         <v>0.2780301406560169</v>
       </c>
       <c r="AK72" t="n">
-        <v>-1.360218025722299</v>
+        <v>3.672198226787098</v>
       </c>
       <c r="AL72" t="n">
-        <v>-29.51261541691159</v>
+        <v>38.08799352038891</v>
       </c>
       <c r="AM72" t="n">
         <v>71</v>
@@ -11410,10 +11410,10 @@
         <v>-0.694697140925294</v>
       </c>
       <c r="AQ72" t="n">
-        <v>-1.15048273565168</v>
+        <v>3.994674560070275</v>
       </c>
       <c r="AR72" t="n">
-        <v>-31.00769214561594</v>
+        <v>45.10967781392873</v>
       </c>
       <c r="AS72" t="n">
         <v>70</v>
@@ -11540,10 +11540,10 @@
         <v>0.2689182997551546</v>
       </c>
       <c r="AK73" t="n">
-        <v>-1.400173751953818</v>
+        <v>3.632242500555579</v>
       </c>
       <c r="AL73" t="n">
-        <v>-30.37953377828829</v>
+        <v>37.67357323373134</v>
       </c>
       <c r="AM73" t="n">
         <v>72</v>
@@ -11558,10 +11558,10 @@
         <v>0.1418970368241607</v>
       </c>
       <c r="AQ73" t="n">
-        <v>-1.8239747796002</v>
+        <v>3.321182516121755</v>
       </c>
       <c r="AR73" t="n">
-        <v>-49.15958031753894</v>
+        <v>37.50430004011889</v>
       </c>
       <c r="AS73" t="n">
         <v>89</v>
@@ -11692,10 +11692,10 @@
         <v>0.2553875552335378</v>
       </c>
       <c r="AK74" t="n">
-        <v>-1.404555885003086</v>
+        <v>3.627860367506312</v>
       </c>
       <c r="AL74" t="n">
-        <v>-30.47461280601996</v>
+        <v>37.62812180521954</v>
       </c>
       <c r="AM74" t="n">
         <v>73</v>
@@ -11710,10 +11710,10 @@
         <v>-0.5535190114692052</v>
       </c>
       <c r="AQ74" t="n">
-        <v>-1.334819258666566</v>
+        <v>3.81033803705539</v>
       </c>
       <c r="AR74" t="n">
-        <v>-35.9759111198895</v>
+        <v>43.02806614882352</v>
       </c>
       <c r="AS74" t="n">
         <v>74</v>
@@ -11840,10 +11840,10 @@
         <v>0.2845914274540443</v>
       </c>
       <c r="AK75" t="n">
-        <v>-1.413442899675329</v>
+        <v>3.618973352834068</v>
       </c>
       <c r="AL75" t="n">
-        <v>-30.66743413412073</v>
+        <v>37.53594580154336</v>
       </c>
       <c r="AM75" t="n">
         <v>74</v>
@@ -11858,10 +11858,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ75" t="n">
-        <v>-1.025385742066247</v>
+        <v>4.119771553655708</v>
       </c>
       <c r="AR75" t="n">
-        <v>-27.63609086448764</v>
+        <v>46.5223298313263</v>
       </c>
       <c r="AS75" t="n">
         <v>66</v>
@@ -11988,10 +11988,10 @@
         <v>0.2130117687666373</v>
       </c>
       <c r="AK76" t="n">
-        <v>-1.464060814586798</v>
+        <v>3.568355437922599</v>
       </c>
       <c r="AL76" t="n">
-        <v>-31.7656897282523</v>
+        <v>37.01093742887432</v>
       </c>
       <c r="AM76" t="n">
         <v>75</v>
@@ -12006,10 +12006,10 @@
         <v>-0.6190486848121851</v>
       </c>
       <c r="AQ76" t="n">
-        <v>-1.42592827904237</v>
+        <v>3.719229016679585</v>
       </c>
       <c r="AR76" t="n">
-        <v>-38.43147204919049</v>
+        <v>41.99922174778602</v>
       </c>
       <c r="AS76" t="n">
         <v>77</v>
@@ -12140,10 +12140,10 @@
         <v>0.3029152054080604</v>
       </c>
       <c r="AK77" t="n">
-        <v>-1.484501501464111</v>
+        <v>3.547914751045287</v>
       </c>
       <c r="AL77" t="n">
-        <v>-32.20919078415642</v>
+        <v>36.79892688334978</v>
       </c>
       <c r="AM77" t="n">
         <v>76</v>
@@ -12158,10 +12158,10 @@
         <v>-0.893676538683964</v>
       </c>
       <c r="AQ77" t="n">
-        <v>-1.147380029029834</v>
+        <v>3.997777266692122</v>
       </c>
       <c r="AR77" t="n">
-        <v>-30.92406831644663</v>
+        <v>45.1447149850319</v>
       </c>
       <c r="AS77" t="n">
         <v>69</v>
@@ -12286,10 +12286,10 @@
         <v>0.2130117687666373</v>
       </c>
       <c r="AK78" t="n">
-        <v>-1.594845861849298</v>
+        <v>3.437570390660099</v>
       </c>
       <c r="AL78" t="n">
-        <v>-34.60332952507176</v>
+        <v>35.65443657432863</v>
       </c>
       <c r="AM78" t="n">
         <v>77</v>
@@ -12304,10 +12304,10 @@
         <v>-0.2133614842544465</v>
       </c>
       <c r="AQ78" t="n">
-        <v>-1.872359002882243</v>
+        <v>3.272798292839712</v>
       </c>
       <c r="AR78" t="n">
-        <v>-50.46362691792925</v>
+        <v>36.95792343528936</v>
       </c>
       <c r="AS78" t="n">
         <v>90</v>
@@ -12434,10 +12434,10 @@
         <v>0.197354844233031</v>
       </c>
       <c r="AK79" t="n">
-        <v>-1.597858984828954</v>
+        <v>3.434557267680444</v>
       </c>
       <c r="AL79" t="n">
-        <v>-34.66870517663704</v>
+        <v>35.62318450092799</v>
       </c>
       <c r="AM79" t="n">
         <v>78</v>
@@ -12452,10 +12452,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ79" t="n">
-        <v>-1.606290726982164</v>
+        <v>3.538866568739791</v>
       </c>
       <c r="AR79" t="n">
-        <v>-43.29258216152862</v>
+        <v>39.96248714176283</v>
       </c>
       <c r="AS79" t="n">
         <v>82</v>
@@ -12582,10 +12582,10 @@
         <v>0.2787364773941335</v>
       </c>
       <c r="AK80" t="n">
-        <v>-1.606941107883499</v>
+        <v>3.425475144625898</v>
       </c>
       <c r="AL80" t="n">
-        <v>-34.86575976627572</v>
+        <v>35.52898483558052</v>
       </c>
       <c r="AM80" t="n">
         <v>79</v>
@@ -12600,10 +12600,10 @@
         <v>-1.573991593113482</v>
       </c>
       <c r="AQ80" t="n">
-        <v>-0.8645821288974833</v>
+        <v>4.280575166824472</v>
       </c>
       <c r="AR80" t="n">
-        <v>-23.30212845155722</v>
+        <v>48.33819719981375</v>
       </c>
       <c r="AS80" t="n">
         <v>57</v>
@@ -12730,10 +12730,10 @@
         <v>0.2450030567271742</v>
       </c>
       <c r="AK81" t="n">
-        <v>-1.607347595597583</v>
+        <v>3.425068656911813</v>
       </c>
       <c r="AL81" t="n">
-        <v>-34.87457931972276</v>
+        <v>35.52476875015593</v>
       </c>
       <c r="AM81" t="n">
         <v>80</v>
@@ -12748,10 +12748,10 @@
         <v>-1.233834065898723</v>
       </c>
       <c r="AQ81" t="n">
-        <v>-1.079662888857127</v>
+        <v>4.065494406864828</v>
       </c>
       <c r="AR81" t="n">
-        <v>-29.09896293208166</v>
+        <v>45.90940766017631</v>
       </c>
       <c r="AS81" t="n">
         <v>67</v>
@@ -12878,10 +12878,10 @@
         <v>0.275210560153981</v>
       </c>
       <c r="AK82" t="n">
-        <v>-1.648239887705943</v>
+        <v>3.384176364803455</v>
       </c>
       <c r="AL82" t="n">
-        <v>-35.76181832677031</v>
+        <v>35.10063441408014</v>
       </c>
       <c r="AM82" t="n">
         <v>81</v>
@@ -12896,10 +12896,10 @@
         <v>-1.573991593113482</v>
       </c>
       <c r="AQ82" t="n">
-        <v>-0.9250975759550126</v>
+        <v>4.220059719766943</v>
       </c>
       <c r="AR82" t="n">
-        <v>-24.93313454514392</v>
+        <v>47.65482931127092</v>
       </c>
       <c r="AS82" t="n">
         <v>64</v>
@@ -13024,10 +13024,10 @@
         <v>0.334387040154814</v>
       </c>
       <c r="AK83" t="n">
-        <v>-1.732746428480897</v>
+        <v>3.2996698240285</v>
       </c>
       <c r="AL83" t="n">
-        <v>-37.59535456209582</v>
+        <v>34.22413364296489</v>
       </c>
       <c r="AM83" t="n">
         <v>82</v>
@@ -13042,10 +13042,10 @@
         <v>-0.694697140925294</v>
       </c>
       <c r="AQ83" t="n">
-        <v>-1.706135879048041</v>
+        <v>3.439021416673914</v>
       </c>
       <c r="AR83" t="n">
-        <v>-45.98359841196999</v>
+        <v>38.8349903774469</v>
       </c>
       <c r="AS83" t="n">
         <v>87</v>
@@ -13172,10 +13172,10 @@
         <v>0.3079495933067176</v>
       </c>
       <c r="AK84" t="n">
-        <v>-1.767281521423187</v>
+        <v>3.26513473108621</v>
       </c>
       <c r="AL84" t="n">
-        <v>-38.34466158282279</v>
+        <v>33.86593609616121</v>
       </c>
       <c r="AM84" t="n">
         <v>83</v>
@@ -13190,10 +13190,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ84" t="n">
-        <v>-1.399953370353322</v>
+        <v>3.745203925368634</v>
       </c>
       <c r="AR84" t="n">
-        <v>-37.7313989866562</v>
+        <v>42.29254220345503</v>
       </c>
       <c r="AS84" t="n">
         <v>76</v>
@@ -13320,10 +13320,10 @@
         <v>0.285613434354803</v>
       </c>
       <c r="AK85" t="n">
-        <v>-1.839647623793299</v>
+        <v>3.192768628716098</v>
       </c>
       <c r="AL85" t="n">
-        <v>-39.91478703924429</v>
+        <v>33.11535579849025</v>
       </c>
       <c r="AM85" t="n">
         <v>84</v>
@@ -13338,10 +13338,10 @@
         <v>-1.233834065898723</v>
       </c>
       <c r="AQ85" t="n">
-        <v>-1.378744199382242</v>
+        <v>3.766413096339714</v>
       </c>
       <c r="AR85" t="n">
-        <v>-37.15977159603529</v>
+        <v>42.53204578624229</v>
       </c>
       <c r="AS85" t="n">
         <v>75</v>
@@ -13472,10 +13472,10 @@
         <v>0.250142386099971</v>
       </c>
       <c r="AK86" t="n">
-        <v>-1.840137925947063</v>
+        <v>3.192278326562334</v>
       </c>
       <c r="AL86" t="n">
-        <v>-39.92542511242704</v>
+        <v>33.11027039075834</v>
       </c>
       <c r="AM86" t="n">
         <v>85</v>
@@ -13490,10 +13490,10 @@
         <v>-0.893676538683964</v>
       </c>
       <c r="AQ86" t="n">
-        <v>-1.607301891002756</v>
+        <v>3.5378554047192</v>
       </c>
       <c r="AR86" t="n">
-        <v>-43.31983495002133</v>
+        <v>39.95106861880183</v>
       </c>
       <c r="AS86" t="n">
         <v>83</v>
@@ -13622,10 +13622,10 @@
         <v>0.2536071876766605</v>
       </c>
       <c r="AK87" t="n">
-        <v>-1.849312921910061</v>
+        <v>3.183103330599336</v>
       </c>
       <c r="AL87" t="n">
-        <v>-40.12449476316475</v>
+        <v>33.01510744878013</v>
       </c>
       <c r="AM87" t="n">
         <v>86</v>
@@ -13640,10 +13640,10 @@
         <v>-0.397239888149268</v>
       </c>
       <c r="AQ87" t="n">
-        <v>-2.0239373032199</v>
+        <v>3.121219992502056</v>
       </c>
       <c r="AR87" t="n">
-        <v>-54.54894965001132</v>
+        <v>35.24623248550287</v>
       </c>
       <c r="AS87" t="n">
         <v>94</v>
@@ -13768,10 +13768,10 @@
         <v>0.3016734153869042</v>
       </c>
       <c r="AK88" t="n">
-        <v>-1.867737293161282</v>
+        <v>3.164678959348115</v>
       </c>
       <c r="AL88" t="n">
-        <v>-40.52424787094094</v>
+        <v>32.82401010340406</v>
       </c>
       <c r="AM88" t="n">
         <v>87</v>
@@ -13786,10 +13786,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ88" t="n">
-        <v>-1.61975962811781</v>
+        <v>3.525397667604145</v>
       </c>
       <c r="AR88" t="n">
-        <v>-43.65559459710182</v>
+        <v>39.81039019829468</v>
       </c>
       <c r="AS88" t="n">
         <v>84</v>
@@ -13914,10 +13914,10 @@
         <v>0.3568994151582677</v>
       </c>
       <c r="AK89" t="n">
-        <v>-1.889287381219383</v>
+        <v>3.143128871290014</v>
       </c>
       <c r="AL89" t="n">
-        <v>-40.99181957564732</v>
+        <v>32.60049286287673</v>
       </c>
       <c r="AM89" t="n">
         <v>88</v>
@@ -13932,10 +13932,10 @@
         <v>-0.4957177431666238</v>
       </c>
       <c r="AQ89" t="n">
-        <v>-1.98942032996618</v>
+        <v>3.155736965755775</v>
       </c>
       <c r="AR89" t="n">
-        <v>-53.61865174350381</v>
+        <v>35.63601381040757</v>
       </c>
       <c r="AS89" t="n">
         <v>93</v>
@@ -14066,10 +14066,10 @@
         <v>0.3145472916259918</v>
       </c>
       <c r="AK90" t="n">
-        <v>-1.919519225265751</v>
+        <v>3.112897027243646</v>
       </c>
       <c r="AL90" t="n">
-        <v>-41.64775911608292</v>
+        <v>32.28692855914498</v>
       </c>
       <c r="AM90" t="n">
         <v>89</v>
@@ -14084,10 +14084,10 @@
         <v>-1.573991593113482</v>
       </c>
       <c r="AQ90" t="n">
-        <v>-1.196623802505679</v>
+        <v>3.948533493216277</v>
       </c>
       <c r="AR90" t="n">
-        <v>-32.25128142509229</v>
+        <v>44.58863194937196</v>
       </c>
       <c r="AS90" t="n">
         <v>71</v>
@@ -14212,10 +14212,10 @@
         <v>0.1561399639256613</v>
       </c>
       <c r="AK91" t="n">
-        <v>-1.939478289815724</v>
+        <v>3.092937962693673</v>
       </c>
       <c r="AL91" t="n">
-        <v>-42.08081042477432</v>
+        <v>32.07991339430255</v>
       </c>
       <c r="AM91" t="n">
         <v>90</v>
@@ -14230,10 +14230,10 @@
         <v>-0.05708236093450922</v>
       </c>
       <c r="AQ91" t="n">
-        <v>-2.407858743977009</v>
+        <v>2.737298551744947</v>
       </c>
       <c r="AR91" t="n">
-        <v>-64.89636076205601</v>
+        <v>30.91081736269801</v>
       </c>
       <c r="AS91" t="n">
         <v>98</v>
@@ -14358,10 +14358,10 @@
         <v>0.2556658361421092</v>
       </c>
       <c r="AK92" t="n">
-        <v>-1.956055890984333</v>
+        <v>3.076360361525064</v>
       </c>
       <c r="AL92" t="n">
-        <v>-42.440494209706</v>
+        <v>31.90797072484432</v>
       </c>
       <c r="AM92" t="n">
         <v>91</v>
@@ -14376,10 +14376,10 @@
         <v>-0.4440127467713617</v>
       </c>
       <c r="AQ92" t="n">
-        <v>-2.105838930442376</v>
+        <v>3.03931836527958</v>
       </c>
       <c r="AR92" t="n">
-        <v>-56.75635386777302</v>
+        <v>34.32136214603337</v>
       </c>
       <c r="AS92" t="n">
         <v>95</v>
@@ -14508,10 +14508,10 @@
         <v>0.2635909872827298</v>
       </c>
       <c r="AK93" t="n">
-        <v>-1.963067315511929</v>
+        <v>3.069348936997468</v>
       </c>
       <c r="AL93" t="n">
-        <v>-42.5926209068197</v>
+        <v>31.83524831840456</v>
       </c>
       <c r="AM93" t="n">
         <v>92</v>
@@ -14526,10 +14526,10 @@
         <v>-0.7841702739861206</v>
       </c>
       <c r="AQ93" t="n">
-        <v>-1.908229189954251</v>
+        <v>3.236928105767705</v>
       </c>
       <c r="AR93" t="n">
-        <v>-51.43039650383222</v>
+        <v>36.55286100589456</v>
       </c>
       <c r="AS93" t="n">
         <v>92</v>
@@ -14656,10 +14656,10 @@
         <v>0.2390842239032407</v>
       </c>
       <c r="AK94" t="n">
-        <v>-1.96631128497851</v>
+        <v>3.066104967530888</v>
       </c>
       <c r="AL94" t="n">
-        <v>-42.66300522865704</v>
+        <v>31.80160190816391</v>
       </c>
       <c r="AM94" t="n">
         <v>93</v>
@@ -14674,10 +14674,10 @@
         <v>-1.233834065898723</v>
       </c>
       <c r="AQ94" t="n">
-        <v>-1.493747674972982</v>
+        <v>3.651409620748974</v>
       </c>
       <c r="AR94" t="n">
-        <v>-40.25933342020607</v>
+        <v>41.2333743542223</v>
       </c>
       <c r="AS94" t="n">
         <v>80</v>
@@ -14808,10 +14808,10 @@
         <v>0.2401585864939016</v>
       </c>
       <c r="AK95" t="n">
-        <v>-1.990575070715115</v>
+        <v>3.041841181794283</v>
       </c>
       <c r="AL95" t="n">
-        <v>-43.18945596189337</v>
+        <v>31.54993822966895</v>
       </c>
       <c r="AM95" t="n">
         <v>94</v>
@@ -14826,10 +14826,10 @@
         <v>-1.034854668140053</v>
       </c>
       <c r="AQ95" t="n">
-        <v>-1.694627377169026</v>
+        <v>3.450529918552929</v>
       </c>
       <c r="AR95" t="n">
-        <v>-45.67342245516208</v>
+        <v>38.96494960292989</v>
       </c>
       <c r="AS95" t="n">
         <v>86</v>
@@ -14954,10 +14954,10 @@
         <v>0.1844207424131122</v>
       </c>
       <c r="AK96" t="n">
-        <v>-2.114900766125589</v>
+        <v>2.917515486383808</v>
       </c>
       <c r="AL96" t="n">
-        <v>-45.8869473682001</v>
+        <v>30.26043369076092</v>
       </c>
       <c r="AM96" t="n">
         <v>95</v>
@@ -14972,10 +14972,10 @@
         <v>-0.5535190114692052</v>
       </c>
       <c r="AQ96" t="n">
-        <v>-2.271641683020905</v>
+        <v>2.87351561270105</v>
       </c>
       <c r="AR96" t="n">
-        <v>-61.22505257096443</v>
+        <v>32.44904222684865</v>
       </c>
       <c r="AS96" t="n">
         <v>97</v>
@@ -15102,10 +15102,10 @@
         <v>0.2272963983911518</v>
       </c>
       <c r="AK97" t="n">
-        <v>-2.179280471261277</v>
+        <v>2.853135781248121</v>
       </c>
       <c r="AL97" t="n">
-        <v>-47.28379216983753</v>
+        <v>29.59268820410237</v>
       </c>
       <c r="AM97" t="n">
         <v>96</v>
@@ -15120,10 +15120,10 @@
         <v>-0.6190486848121851</v>
       </c>
       <c r="AQ97" t="n">
-        <v>-2.191790634731098</v>
+        <v>2.953366660990858</v>
       </c>
       <c r="AR97" t="n">
-        <v>-59.07291534530449</v>
+        <v>33.35075649850995</v>
       </c>
       <c r="AS97" t="n">
         <v>96</v>
@@ -15248,10 +15248,10 @@
         <v>0.334387040154814</v>
       </c>
       <c r="AK98" t="n">
-        <v>-2.220060209647354</v>
+        <v>2.812356042862044</v>
       </c>
       <c r="AL98" t="n">
-        <v>-48.16858910167607</v>
+        <v>29.16972127380923</v>
       </c>
       <c r="AM98" t="n">
         <v>97</v>
@@ -15266,10 +15266,10 @@
         <v>-1.573991593113482</v>
       </c>
       <c r="AQ98" t="n">
-        <v>-1.689673262751974</v>
+        <v>3.455484032969981</v>
       </c>
       <c r="AR98" t="n">
-        <v>-45.53989967386534</v>
+        <v>39.02089371097824</v>
       </c>
       <c r="AS98" t="n">
         <v>85</v>
@@ -15394,10 +15394,10 @@
         <v>0.1536622743292751</v>
       </c>
       <c r="AK99" t="n">
-        <v>-2.266723699738118</v>
+        <v>2.765692552771279</v>
       </c>
       <c r="AL99" t="n">
-        <v>-49.18104564247825</v>
+        <v>28.68572814531986</v>
       </c>
       <c r="AM99" t="n">
         <v>98</v>
@@ -15412,10 +15412,10 @@
         <v>-0.6190486848121851</v>
       </c>
       <c r="AQ99" t="n">
-        <v>-2.422710389290367</v>
+        <v>2.722446906431588</v>
       </c>
       <c r="AR99" t="n">
-        <v>-65.29664077622905</v>
+        <v>30.74310584452103</v>
       </c>
       <c r="AS99" t="n">
         <v>99</v>
@@ -15544,10 +15544,10 @@
         <v>0.2370040327832862</v>
       </c>
       <c r="AK100" t="n">
-        <v>-2.369485750798467</v>
+        <v>2.66293050171093</v>
       </c>
       <c r="AL100" t="n">
-        <v>-51.41067121356026</v>
+        <v>27.61988145262841</v>
       </c>
       <c r="AM100" t="n">
         <v>99</v>
@@ -15562,10 +15562,10 @@
         <v>-1.573991593113482</v>
       </c>
       <c r="AQ100" t="n">
-        <v>-1.880451720619214</v>
+        <v>3.264705575102742</v>
       </c>
       <c r="AR100" t="n">
-        <v>-50.68174101250297</v>
+        <v>36.8665367943342</v>
       </c>
       <c r="AS100" t="n">
         <v>91</v>

</xml_diff>